<commit_message>
Updated the software process model
</commit_message>
<xml_diff>
--- a/Bes(t)Poke SE216_SoftwareProcessModel.xlsx
+++ b/Bes(t)Poke SE216_SoftwareProcessModel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\SE 216 PROJECT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62809C4-59A6-4E4D-AA61-4A326BCA74FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE90341-7281-411F-84FA-F1A16578549B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DD0626E2-1333-F643-A88B-8507C5CC965E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{DD0626E2-1333-F643-A88B-8507C5CC965E}"/>
   </bookViews>
   <sheets>
     <sheet name="ProductBackLog" sheetId="4" r:id="rId1"/>
@@ -191,9 +191,6 @@
     <t>Both the clients and creators can post reviews and ratings after the comission process is finished.</t>
   </si>
   <si>
-    <t>Allow access to different permission sets according to the chosen role.</t>
-  </si>
-  <si>
     <t>Creator-defined order forms with multiple field types(e.g., text input, multiple choice,
 checkbox, dropdown list, and file upload (max 20MB))</t>
   </si>
@@ -362,6 +359,9 @@
   </si>
   <si>
     <t>Naz,Aslı,Zeynep</t>
+  </si>
+  <si>
+    <t>Allow access to different permission sets according to the chosen role, let the creators upload their portfolios</t>
   </si>
 </sst>
 </file>
@@ -18011,7 +18011,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="91.95" customHeight="1">
       <c r="A1" s="72" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="73"/>
     </row>
@@ -18036,7 +18036,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" customHeight="1">
@@ -18052,7 +18052,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" customHeight="1">
@@ -18068,7 +18068,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" customHeight="1">
@@ -18076,7 +18076,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="45" customHeight="1">
@@ -18084,7 +18084,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="45" customHeight="1">
@@ -18092,7 +18092,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="45" customHeight="1">
@@ -18100,7 +18100,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="45" customHeight="1">
@@ -18124,7 +18124,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45" customHeight="1">
@@ -18132,7 +18132,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="45" customHeight="1">
@@ -18156,7 +18156,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="45" customHeight="1">
@@ -18164,7 +18164,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="45" customHeight="1">
@@ -18254,7 +18254,7 @@
     <row r="3" spans="1:15" ht="46.05" customHeight="1">
       <c r="A3" s="62"/>
       <c r="B3" s="56" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="39" t="s">
         <v>34</v>
@@ -18282,7 +18282,7 @@
     <row r="4" spans="1:15" ht="22.05" customHeight="1">
       <c r="A4" s="62"/>
       <c r="B4" s="56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>25</v>
@@ -18303,17 +18303,17 @@
         <v>1</v>
       </c>
       <c r="I4" s="39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:15" ht="22.05" customHeight="1">
       <c r="A5" s="62"/>
       <c r="B5" s="56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5" s="61" t="s">
         <v>18</v>
@@ -18331,14 +18331,14 @@
         <v>1</v>
       </c>
       <c r="I5" s="56" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="M5" s="3"/>
     </row>
     <row r="6" spans="1:15" ht="22.05" customHeight="1">
       <c r="A6" s="58"/>
       <c r="B6" s="56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6" s="56" t="s">
         <v>32</v>
@@ -18859,7 +18859,7 @@
     <row r="3" spans="1:15" ht="22.05" customHeight="1">
       <c r="A3" s="62"/>
       <c r="B3" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C3" s="39" t="s">
         <v>41</v>
@@ -18880,14 +18880,14 @@
         <v>2</v>
       </c>
       <c r="I3" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M3" s="3"/>
     </row>
     <row r="4" spans="1:15" ht="22.05" customHeight="1">
       <c r="A4" s="62"/>
       <c r="B4" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="56" t="s">
         <v>42</v>
@@ -18915,10 +18915,10 @@
     <row r="5" spans="1:15" ht="22.05" customHeight="1">
       <c r="A5" s="62"/>
       <c r="B5" s="71" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5" s="57" t="s">
         <v>27</v>
@@ -18936,17 +18936,17 @@
         <v>1</v>
       </c>
       <c r="I5" s="56" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M5" s="3"/>
     </row>
     <row r="6" spans="1:15" ht="22.05" customHeight="1">
       <c r="A6" s="62"/>
       <c r="B6" s="56" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C6" s="56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6" s="57" t="s">
         <v>27</v>
@@ -18964,17 +18964,17 @@
         <v>1</v>
       </c>
       <c r="I6" s="56" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:15" ht="21.6" customHeight="1">
       <c r="A7" s="62"/>
       <c r="B7" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7" s="57" t="s">
         <v>27</v>
@@ -18992,17 +18992,17 @@
         <v>2</v>
       </c>
       <c r="I7" s="56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M7" s="3"/>
     </row>
     <row r="8" spans="1:15" ht="21.6" customHeight="1">
       <c r="A8" s="62"/>
       <c r="B8" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C8" s="56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" s="57" t="s">
         <v>27</v>
@@ -19020,7 +19020,7 @@
         <v>2</v>
       </c>
       <c r="I8" s="56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M8" s="3"/>
     </row>
@@ -19475,10 +19475,10 @@
     <row r="3" spans="1:15" ht="22.05" customHeight="1">
       <c r="A3" s="62"/>
       <c r="B3" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C3" s="56" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" s="57" t="s">
         <v>27</v>
@@ -19496,17 +19496,17 @@
         <v>2</v>
       </c>
       <c r="I3" s="56" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M3" s="3"/>
     </row>
     <row r="4" spans="1:15" ht="22.05" customHeight="1">
       <c r="A4" s="62"/>
       <c r="B4" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>27</v>
@@ -19532,10 +19532,10 @@
     <row r="5" spans="1:15" s="69" customFormat="1" ht="22.05" customHeight="1">
       <c r="A5"/>
       <c r="B5" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" s="57" t="s">
         <v>27</v>
@@ -20057,10 +20057,10 @@
     <row r="3" spans="1:15" ht="22.05" customHeight="1">
       <c r="A3" s="58"/>
       <c r="B3" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C3" s="56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" s="57" t="s">
         <v>27</v>
@@ -20085,10 +20085,10 @@
     <row r="4" spans="1:15" ht="22.05" customHeight="1">
       <c r="A4" s="58"/>
       <c r="B4" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>27</v>
@@ -20106,16 +20106,16 @@
         <v>2</v>
       </c>
       <c r="I4" s="56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:15" s="69" customFormat="1" ht="22.05" customHeight="1">
       <c r="B5" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D5" s="66" t="s">
         <v>27</v>
@@ -20133,16 +20133,16 @@
         <v>1</v>
       </c>
       <c r="I5" s="65" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M5" s="68"/>
     </row>
     <row r="6" spans="1:15" s="69" customFormat="1" ht="22.05" customHeight="1">
       <c r="B6" s="56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D6" s="66" t="s">
         <v>27</v>
@@ -20160,7 +20160,7 @@
         <v>3</v>
       </c>
       <c r="I6" s="65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M6" s="68"/>
     </row>

</xml_diff>